<commit_message>
increase Pads for Handsolder, fix issue with rectifier
</commit_message>
<xml_diff>
--- a/io-gateway/bom1.xlsx
+++ b/io-gateway/bom1.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\baischerl\Documents\localProject\cad\RS485-IO-Extension\io-gateway\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{199A55BB-7C25-435D-9956-545AEF6916F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B48BC4-96CF-40BB-8E7D-22E76EA9695E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F15727DA-6B17-406F-B179-A37C389DC2DE}"/>
+    <workbookView xWindow="-4800" yWindow="-2340" windowWidth="38640" windowHeight="21120" xr2:uid="{F15727DA-6B17-406F-B179-A37C389DC2DE}"/>
   </bookViews>
   <sheets>
     <sheet name="bom1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="167">
   <si>
     <t>Id</t>
   </si>
@@ -55,9 +68,6 @@
     <t>C_1210_3225Metric</t>
   </si>
   <si>
-    <t>10ÂµF 50V</t>
-  </si>
-  <si>
     <t>GRM32EC72A106ME05K Murata Electronics | Mouser Österreich</t>
   </si>
   <si>
@@ -67,9 +77,6 @@
     <t>D_SMB</t>
   </si>
   <si>
-    <t>D_Schottky</t>
-  </si>
-  <si>
     <t>STPS3L60UF STMicroelectronics | Mouser Österreich</t>
   </si>
   <si>
@@ -130,9 +137,6 @@
     <t>D_DIMA_2,D_DIMA_8,D_DIMB_2,D_DIMB_6,D_DIMB_10,D_DIMB_8,D_DIMA_6,D_DIMA_10</t>
   </si>
   <si>
-    <t>D_Zener</t>
-  </si>
-  <si>
     <t>https://www.mouser.at/ProductDetail/863-MMSZ39T1G</t>
   </si>
   <si>
@@ -154,9 +158,6 @@
     <t>TerminalBlock_MaiXu_MX126-5.0-02P_1x02_P5.00mm</t>
   </si>
   <si>
-    <t>Screw_Terminal_01x02</t>
-  </si>
-  <si>
     <t>1-282836-3 TE Connectivity | Mouser Österreich</t>
   </si>
   <si>
@@ -328,24 +329,15 @@
     <t>HSOP-8-1EP_3.9x4.9mm_P1.27mm_EP2.41x3.1mm</t>
   </si>
   <si>
-    <t>LED5000</t>
-  </si>
-  <si>
     <t>U6</t>
   </si>
   <si>
     <t>SOT-23</t>
   </si>
   <si>
-    <t>MCP9700x-ETT</t>
-  </si>
-  <si>
     <t>C41,C42</t>
   </si>
   <si>
-    <t>22ÂµF</t>
-  </si>
-  <si>
     <t>U3</t>
   </si>
   <si>
@@ -364,9 +356,6 @@
     <t>R_1206_3216Metric</t>
   </si>
   <si>
-    <t>1 || 0,5 || 0,25</t>
-  </si>
-  <si>
     <t>AC1206FR-7W1RL YAGEO | Mouser Österreich</t>
   </si>
   <si>
@@ -394,9 +383,6 @@
     <t>R4,R3</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
     <t>Reserve</t>
   </si>
   <si>
@@ -421,9 +407,6 @@
     <t>C10,C11</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -442,9 +425,6 @@
     <t>R30</t>
   </si>
   <si>
-    <t>49.9</t>
-  </si>
-  <si>
     <t>U2</t>
   </si>
   <si>
@@ -484,12 +464,6 @@
     <t>47µH  3.8A</t>
   </si>
   <si>
-    <t>47 µF</t>
-  </si>
-  <si>
-    <t>1 µF 50V</t>
-  </si>
-  <si>
     <t>https://www.mouser.at/ProductDetail/Vishay-Draloric/RCA0603100KFKEAHP?qs=rrS6PyfT74exmGMHOWeh9Q%3D%3D</t>
   </si>
   <si>
@@ -527,6 +501,39 @@
   </si>
   <si>
     <t>Quantitiy ordered</t>
+  </si>
+  <si>
+    <t>STPS3L60UF</t>
+  </si>
+  <si>
+    <t>1 µF 100V</t>
+  </si>
+  <si>
+    <t>MMSZ39T1G</t>
+  </si>
+  <si>
+    <t>1-282836-3</t>
+  </si>
+  <si>
+    <t>10µF 100V</t>
+  </si>
+  <si>
+    <t>100R</t>
+  </si>
+  <si>
+    <t>LED5000PHR</t>
+  </si>
+  <si>
+    <t>MCP9700T-E/LT</t>
+  </si>
+  <si>
+    <t>22µF</t>
+  </si>
+  <si>
+    <t>47µF</t>
+  </si>
+  <si>
+    <t>49.9R</t>
   </si>
 </sst>
 </file>
@@ -534,7 +541,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="_-[$€-C07]\ * #,##0.00_-;\-[$€-C07]\ * #,##0.00_-;_-[$€-C07]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-[$€-C07]\ * #,##0.00_-;\-[$€-C07]\ * #,##0.00_-;_-[$€-C07]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -1025,8 +1032,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="0" xfId="6" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="6" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1440,7 +1447,7 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>7</v>
@@ -1463,7 +1470,7 @@
         <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>160</v>
       </c>
       <c r="F2" s="2">
         <v>0.39900000000000002</v>
@@ -1480,7 +1487,7 @@
         <v>6.7830000000000004</v>
       </c>
       <c r="J2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1488,16 +1495,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
       </c>
       <c r="D3">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>156</v>
       </c>
       <c r="F3" s="2">
         <v>0.14199999999999999</v>
@@ -1514,7 +1521,7 @@
         <v>14.2</v>
       </c>
       <c r="J3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1522,7 +1529,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C4">
         <v>20715562</v>
@@ -1531,7 +1538,7 @@
         <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F4" s="2">
         <v>1.24</v>
@@ -1548,7 +1555,7 @@
         <v>12.4</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1556,16 +1563,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F5" s="2">
         <v>0.152</v>
@@ -1582,7 +1589,7 @@
         <v>1.52</v>
       </c>
       <c r="J5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1590,16 +1597,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="F6" s="2">
         <v>0</v>
@@ -1616,7 +1623,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1624,16 +1631,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D7">
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F7" s="2">
         <v>4.2000000000000003E-2</v>
@@ -1650,7 +1657,7 @@
         <v>4.2</v>
       </c>
       <c r="J7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1658,7 +1665,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8">
         <v>1752201</v>
@@ -1684,7 +1691,7 @@
         <v>116.46</v>
       </c>
       <c r="J8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1692,16 +1699,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
         <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>34</v>
       </c>
       <c r="F9" s="2">
         <v>4.2000000000000003E-2</v>
@@ -1718,7 +1725,7 @@
         <v>4.62</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1726,16 +1733,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D10">
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>158</v>
       </c>
       <c r="F10" s="2">
         <v>3.3000000000000002E-2</v>
@@ -1752,10 +1759,10 @@
         <v>4.9400000000000004</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1763,16 +1770,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D11">
         <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F11" s="2">
         <v>2.4E-2</v>
@@ -1789,7 +1796,7 @@
         <v>2.4</v>
       </c>
       <c r="J11" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1797,16 +1804,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D12">
         <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>159</v>
       </c>
       <c r="F12" s="2">
         <v>0.54600000000000004</v>
@@ -1823,24 +1830,24 @@
         <v>54.6</v>
       </c>
       <c r="J12" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>0.495</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D13">
         <v>8</v>
       </c>
       <c r="E13" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="F13" s="2">
         <v>0.495</v>
@@ -1857,7 +1864,7 @@
         <v>49.5</v>
       </c>
       <c r="J13" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1865,16 +1872,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F14" s="2">
         <v>1.33</v>
@@ -1891,7 +1898,7 @@
         <v>1.33</v>
       </c>
       <c r="J14" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1899,16 +1906,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F15" s="2">
         <v>0.28999999999999998</v>
@@ -1925,7 +1932,7 @@
         <v>4.3499999999999996</v>
       </c>
       <c r="J15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1933,16 +1940,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D16">
         <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
@@ -1959,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -1967,16 +1974,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D17">
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F17" s="2">
         <v>3.5000000000000003E-2</v>
@@ -1993,7 +2000,7 @@
         <v>3.5000000000000004</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -2001,16 +2008,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D18">
         <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F18" s="2">
         <v>7.0000000000000001E-3</v>
@@ -2027,7 +2034,7 @@
         <v>0.70000000000000007</v>
       </c>
       <c r="J18" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -2035,16 +2042,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C19" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D19">
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F19" s="2">
         <v>3.0000000000000001E-3</v>
@@ -2061,7 +2068,7 @@
         <v>0.3</v>
       </c>
       <c r="J19" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -2069,16 +2076,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D20">
         <v>18</v>
       </c>
       <c r="E20" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F20" s="2">
         <v>8.0000000000000002E-3</v>
@@ -2095,7 +2102,7 @@
         <v>1.6</v>
       </c>
       <c r="J20" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2103,16 +2110,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D21">
         <v>4</v>
       </c>
       <c r="E21" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="F21" s="2">
         <v>2.8000000000000001E-2</v>
@@ -2129,7 +2136,7 @@
         <v>2.8000000000000003</v>
       </c>
       <c r="J21" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -2137,16 +2144,16 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C22" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="F22" s="2">
         <v>0.69299999999999995</v>
@@ -2163,7 +2170,7 @@
         <v>6.93</v>
       </c>
       <c r="J22" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -2171,16 +2178,16 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D23">
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F23" s="2">
         <v>2.11</v>
@@ -2197,7 +2204,7 @@
         <v>2.11</v>
       </c>
       <c r="J23" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -2205,16 +2212,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D24">
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F24" s="2">
         <v>5.0000000000000001E-3</v>
@@ -2231,7 +2238,7 @@
         <v>0.5</v>
       </c>
       <c r="J24" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -2239,16 +2246,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D25">
         <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F25" s="2">
         <v>8.0000000000000002E-3</v>
@@ -2265,7 +2272,7 @@
         <v>0.8</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -2273,16 +2280,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C26" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D26">
         <v>8</v>
       </c>
       <c r="E26" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F26" s="2">
         <v>2.7E-2</v>
@@ -2299,7 +2306,7 @@
         <v>2.7</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -2307,16 +2314,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D27">
         <v>10</v>
       </c>
-      <c r="E27">
-        <v>100</v>
+      <c r="E27" t="s">
+        <v>161</v>
       </c>
       <c r="F27" s="2">
         <v>6.0000000000000001E-3</v>
@@ -2333,7 +2340,7 @@
         <v>0.72</v>
       </c>
       <c r="J27" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -2341,16 +2348,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D28">
         <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F28" s="2">
         <v>0.16300000000000001</v>
@@ -2367,7 +2374,7 @@
         <v>1.6300000000000001</v>
       </c>
       <c r="J28" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -2375,16 +2382,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F29" s="2">
         <v>12.75</v>
@@ -2401,7 +2408,7 @@
         <v>25.5</v>
       </c>
       <c r="J29" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -2409,16 +2416,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C30" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D30">
         <v>10</v>
       </c>
       <c r="E30" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F30" s="2">
         <v>3.6999999999999998E-2</v>
@@ -2435,7 +2442,7 @@
         <v>3.6999999999999997</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -2443,16 +2450,16 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C31" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D31">
         <v>8</v>
       </c>
       <c r="E31" t="s">
-        <v>102</v>
+        <v>162</v>
       </c>
       <c r="F31" s="2">
         <v>1.39</v>
@@ -2469,7 +2476,7 @@
         <v>13.899999999999999</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -2477,16 +2484,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C32" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D32">
         <v>1</v>
       </c>
       <c r="E32" t="s">
-        <v>105</v>
+        <v>163</v>
       </c>
       <c r="F32" s="2">
         <v>0.34399999999999997</v>
@@ -2503,7 +2510,7 @@
         <v>0.68799999999999994</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
@@ -2511,16 +2518,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C33" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D33">
         <v>2</v>
       </c>
       <c r="E33" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="F33" s="2">
         <v>0</v>
@@ -2537,7 +2544,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
@@ -2545,16 +2552,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C34" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D34">
         <v>1</v>
       </c>
       <c r="E34" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="F34" s="2">
         <v>0.745</v>
@@ -2571,7 +2578,7 @@
         <v>7.45</v>
       </c>
       <c r="J34" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
@@ -2579,16 +2586,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C35" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="D35">
         <v>8</v>
       </c>
       <c r="E35" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F35" s="2">
         <v>0.47</v>
@@ -2605,13 +2612,13 @@
         <v>23.5</v>
       </c>
       <c r="J35" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="K35" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="L35" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
@@ -2619,16 +2626,16 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C36" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D36">
         <v>8</v>
       </c>
       <c r="E36" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="F36" s="2">
         <v>0</v>
@@ -2645,7 +2652,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
@@ -2653,16 +2660,16 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C37" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D37">
         <v>1</v>
       </c>
       <c r="E37" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F37" s="2">
         <v>2.42</v>
@@ -2679,7 +2686,7 @@
         <v>24.2</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
@@ -2687,16 +2694,16 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C38" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D38">
         <v>2</v>
       </c>
       <c r="E38" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="F38" s="2">
         <v>0</v>
@@ -2713,7 +2720,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
@@ -2721,16 +2728,16 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="C39" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D39">
         <v>2</v>
       </c>
       <c r="E39" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="F39" s="2">
         <v>0.114</v>
@@ -2747,7 +2754,7 @@
         <v>2.2800000000000002</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
@@ -2755,16 +2762,16 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="C40" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D40">
         <v>1</v>
       </c>
       <c r="E40" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="F40" s="2">
         <v>0</v>
@@ -2781,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -2789,16 +2796,16 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D41">
         <v>1</v>
       </c>
       <c r="E41" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F41" s="2">
         <v>0</v>
@@ -2815,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
@@ -2823,16 +2830,16 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C42" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D42">
         <v>2</v>
       </c>
       <c r="E42" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="F42" s="2">
         <v>0</v>
@@ -2849,7 +2856,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
@@ -2857,16 +2864,16 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C43" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="F43" s="2">
         <v>2.33</v>
@@ -2883,7 +2890,7 @@
         <v>2.33</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -2891,16 +2898,16 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C44" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D44">
         <v>1</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="F44" s="2">
         <v>3.5999999999999997E-2</v>
@@ -2917,7 +2924,7 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -2925,16 +2932,16 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C45" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D45">
         <v>1</v>
       </c>
       <c r="E45" t="s">
-        <v>140</v>
+        <v>166</v>
       </c>
       <c r="F45" s="2">
         <v>0</v>
@@ -2951,7 +2958,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
@@ -2959,16 +2966,16 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C46" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D46">
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="F46" s="2">
         <v>0.69899999999999995</v>
@@ -2985,7 +2992,7 @@
         <v>6.9899999999999993</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
@@ -2993,10 +3000,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="C47" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -3016,7 +3023,7 @@
         <v>5.96</v>
       </c>
       <c r="J47" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
@@ -3024,10 +3031,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="C48" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="D48">
         <v>2</v>
@@ -3047,7 +3054,7 @@
         <v>5.96</v>
       </c>
       <c r="J48" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
@@ -3055,10 +3062,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="C49" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -3078,7 +3085,7 @@
         <v>2.98</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>